<commit_message>
Add concrete methods and STATIC/DYNAMIC field mapping to NT xlsx
Each workbook now includes start-parameter classification and a Methods
sheet with job types, endpoints, and static vs dynamic inputs per step.

Co-authored-by: Дмитрий Григорьев <pulya-na-vullet@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/nt-prerequisites-xlsx/00-README-index.xlsx
+++ b/nt-prerequisites-xlsx/00-README-index.xlsx
@@ -439,24 +439,25 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B19"/>
+  <dimension ref="A1:C17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
     <col width="45" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>НТ пререквизиты — некредитное страхование (ncins)</t>
+          <t>НТ пререквизиты ncins — Excel</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Табличный формат для специалиста НТ · 21.07.2026</t>
+          <t>В каждом файле: лист «0. Старт STATIC vs DYNAMIC» + «1. Методы» с конкретными endpoint/job type</t>
         </is>
       </c>
     </row>
@@ -472,7 +473,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="30" customHeight="1">
+    <row r="5" ht="35" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
           <t>01-ump-main-ma-ncins-pa.xlsx</t>
@@ -480,11 +481,11 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Управление процессом мультизаявки</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="30" customHeight="1">
+          <t>Управление мультизаявкой</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="35" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
         <is>
           <t>02-ump-prepare-documents-ncins-pa.xlsx</t>
@@ -496,7 +497,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="30" customHeight="1">
+    <row r="7" ht="35" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
           <t>03-ump-signing-documents-ncins-pa.xlsx</t>
@@ -508,7 +509,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="30" customHeight="1">
+    <row r="8" ht="35" customHeight="1">
       <c r="A8" s="3" t="inlineStr">
         <is>
           <t>04-ump-payment-ncins-pa.xlsx</t>
@@ -520,7 +521,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="30" customHeight="1">
+    <row r="9" ht="35" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
         <is>
           <t>05-ump-finalisation-ncins-pa.xlsx</t>
@@ -532,7 +533,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="30" customHeight="1">
+    <row r="10" ht="35" customHeight="1">
       <c r="A10" s="3" t="inlineStr">
         <is>
           <t>06-ump-delete-documents-ncins-pa.xlsx</t>
@@ -547,84 +548,85 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Параметр</t>
+          <t>Тип</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Значение</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="30" customHeight="1">
+          <t>Смысл</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Цвет в Excel</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="35" customHeight="1">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>База</t>
+          <t>STATIC</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>15000 заявок / месяц</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="30" customHeight="1">
+          <t>Константа в BPMN/коннекторе/коде</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>оранжевый</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="35" customHeight="1">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>Канал</t>
+          <t>DYNAMIC_START</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>SFA, рабочие часы ЮЛ</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="30" customHeight="1">
+          <t>Приходит на старте процесса</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>зелёный</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="35" customHeight="1">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>Среднее</t>
+          <t>DYNAMIC_FROM_APP</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>~89 заявок/час</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="30" customHeight="1">
+          <t>Из GET /applications/{id}</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>зелёный</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="35" customHeight="1">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>Пик (×2)</t>
+          <t>DYNAMIC_FROM_PREV</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>~180 заявок/час</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="30" customHeight="1">
-      <c r="A18" s="3" t="inlineStr">
-        <is>
-          <t>Timeout-ветки</t>
-        </is>
-      </c>
-      <c r="B18" s="3" t="inlineStr">
-        <is>
-          <t>~5% (~750/мес, ~4–5/час)</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="30" customHeight="1">
-      <c r="A19" s="3" t="inlineStr">
-        <is>
-          <t>Из timeout: signing</t>
-        </is>
-      </c>
-      <c r="B19" s="3" t="inlineStr">
-        <is>
-          <t>~95%</t>
+          <t>Из предыдущего шага / Kafka message</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>зелёный</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Rebuild NT docs to match onboarding-pa template structure
Six Excel workbooks now use the same prerequisite questions (1-12) and
columns as the sample, filled with SA and backend answers for each ncins worker.

Co-authored-by: Дмитрий Григорьев <pulya-na-vullet@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/nt-prerequisites-xlsx/00-README-index.xlsx
+++ b/nt-prerequisites-xlsx/00-README-index.xlsx
@@ -34,20 +34,15 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00D6EAF8"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -55,25 +50,14 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -439,25 +423,24 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="70" customWidth="1" min="1" max="1"/>
     <col width="45" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>НТ пререквизиты ncins — Excel</t>
+          <t>НТ пререквизиты — пакет ncins (структура = образец ump-onboarding-pa)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>В каждом файле: лист «0. Старт STATIC vs DYNAMIC» + «1. Методы» с конкретными endpoint/job type</t>
+          <t>Одинаковые вопросы (пререквизиты 1–12), ответы — СА + бэкенд. TBD где данных нет.</t>
         </is>
       </c>
     </row>
@@ -473,160 +456,75 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="35" customHeight="1">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>01-ump-main-ma-ncins-pa.xlsx</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>Управление мультизаявкой</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="35" customHeight="1">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>02-ump-prepare-documents-ncins-pa.xlsx</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>Формирование документов</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="35" customHeight="1">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>03-ump-signing-documents-ncins-pa.xlsx</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="inlineStr">
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>НТ пререквизиты __ Worker ump-main-ma-ncins-pa.xlsx</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Управление процессом мультизаявки</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>НТ пререквизиты __ Worker ump-prepare-documents-ncins-pa.xlsx</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Формирования документов</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>НТ пререквизиты __ Worker ump-signing-documents-ncins-pa.xlsx</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
         <is>
           <t>Подписание документов</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="35" customHeight="1">
-      <c r="A8" s="3" t="inlineStr">
-        <is>
-          <t>04-ump-payment-ncins-pa.xlsx</t>
-        </is>
-      </c>
-      <c r="B8" s="3" t="inlineStr">
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>НТ пререквизиты __ Worker ump-payment-ncins-pa.xlsx</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
         <is>
           <t>Оплата страховки</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="35" customHeight="1">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t>05-ump-finalisation-ncins-pa.xlsx</t>
-        </is>
-      </c>
-      <c r="B9" s="3" t="inlineStr">
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>НТ пререквизиты __ Worker ump-finalisation-ncins-pa.xlsx</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
         <is>
           <t>Финализация заявки</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="35" customHeight="1">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>06-ump-delete-documents-ncins-pa.xlsx</t>
-        </is>
-      </c>
-      <c r="B10" s="3" t="inlineStr">
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>НТ пререквизиты __ Worker ump-delete-documents-ncins-pa.xlsx</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
         <is>
           <t>Удаление документов</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>Тип</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>Смысл</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>Цвет в Excel</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="35" customHeight="1">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>STATIC</t>
-        </is>
-      </c>
-      <c r="B14" s="3" t="inlineStr">
-        <is>
-          <t>Константа в BPMN/коннекторе/коде</t>
-        </is>
-      </c>
-      <c r="C14" s="3" t="inlineStr">
-        <is>
-          <t>оранжевый</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="35" customHeight="1">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t>DYNAMIC_START</t>
-        </is>
-      </c>
-      <c r="B15" s="3" t="inlineStr">
-        <is>
-          <t>Приходит на старте процесса</t>
-        </is>
-      </c>
-      <c r="C15" s="3" t="inlineStr">
-        <is>
-          <t>зелёный</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="35" customHeight="1">
-      <c r="A16" s="3" t="inlineStr">
-        <is>
-          <t>DYNAMIC_FROM_APP</t>
-        </is>
-      </c>
-      <c r="B16" s="3" t="inlineStr">
-        <is>
-          <t>Из GET /applications/{id}</t>
-        </is>
-      </c>
-      <c r="C16" s="3" t="inlineStr">
-        <is>
-          <t>зелёный</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="35" customHeight="1">
-      <c r="A17" s="3" t="inlineStr">
-        <is>
-          <t>DYNAMIC_FROM_PREV</t>
-        </is>
-      </c>
-      <c r="B17" s="3" t="inlineStr">
-        <is>
-          <t>Из предыдущего шага / Kafka message</t>
-        </is>
-      </c>
-      <c r="C17" s="3" t="inlineStr">
-        <is>
-          <t>зелёный</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update all 6 NT Excel docs from final BPMN PR
Align prerequisites with NCINS BPMN: correlationKey, timers
PT25M/PT5M/PT30M, finalisation 3× parallel ea-send, delete
multiInstance DELETE_DOCS, main Call Activity cleanup.

Co-authored-by: Дмитрий Григорьев <pulya-na-vullet@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/nt-prerequisites-xlsx/00-README-index.xlsx
+++ b/nt-prerequisites-xlsx/00-README-index.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -26,23 +26,39 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
       <sz val="14"/>
     </font>
     <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
       <b val="1"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D6EAF8"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -50,14 +66,32 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00BFBFBF"/>
+      </left>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -423,11 +457,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="70" customWidth="1" min="1" max="1"/>
-    <col width="45" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -438,91 +472,91 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Одинаковые вопросы (пререквизиты 1–12), ответы — СА + бэкенд. TBD где данных нет.</t>
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Одинаковые вопросы (пререквизиты 1–12). Ответы — СА + бэкенд + сверка с BPMN PR. TBD где данных нет.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Файл</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Процесс</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>Файл</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>Процесс</t>
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>НТ пререквизиты __ Worker ump-main-ma-ncins-pa.xlsx</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Управление процессом мультизаявки</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>НТ пререквизиты __ Worker ump-main-ma-ncins-pa.xlsx</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Управление процессом мультизаявки</t>
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>НТ пререквизиты __ Worker ump-prepare-documents-ncins-pa.xlsx</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Формирования документов</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>НТ пререквизиты __ Worker ump-prepare-documents-ncins-pa.xlsx</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Формирования документов</t>
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>НТ пререквизиты __ Worker ump-signing-documents-ncins-pa.xlsx</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Подписание документов</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>НТ пререквизиты __ Worker ump-signing-documents-ncins-pa.xlsx</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Подписание документов</t>
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>НТ пререквизиты __ Worker ump-payment-ncins-pa.xlsx</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Оплата страховки</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>НТ пререквизиты __ Worker ump-payment-ncins-pa.xlsx</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Оплата страховки</t>
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>НТ пререквизиты __ Worker ump-finalisation-ncins-pa.xlsx</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>Финализация заявки</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>НТ пререквизиты __ Worker ump-finalisation-ncins-pa.xlsx</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Финализация заявки</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A9" s="4" t="inlineStr">
         <is>
           <t>НТ пререквизиты __ Worker ump-delete-documents-ncins-pa.xlsx</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B9" s="4" t="inlineStr">
         <is>
           <t>Удаление документов</t>
         </is>

</xml_diff>

<commit_message>
Fill NT docs from develop workers and IT examples
Map JobWorker types to HTTP/stubs using ump-ncins-pa develop
archive; add concrete request/response from WorkerIT stubs.

Co-authored-by: Дмитрий Григорьев <pulya-na-vullet@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/nt-prerequisites-xlsx/00-README-index.xlsx
+++ b/nt-prerequisites-xlsx/00-README-index.xlsx
@@ -461,20 +461,20 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="70" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="45" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>НТ пререквизиты — пакет ncins (структура = образец ump-onboarding-pa)</t>
+          <t>НТ пререквизиты ncins — по коду develop ump-ncins-pa@4a921a1653e</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Одинаковые вопросы (пререквизиты 1–12). Ответы — СА + бэкенд + сверка с BPMN PR. TBD где данных нет.</t>
+          <t>Примеры request/response из *Worker.java + *WorkerIT + stubs. BPMN main-ma в develop нет.</t>
         </is>
       </c>
     </row>
@@ -498,7 +498,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Управление процессом мультизаявки</t>
+          <t>Оркестратор (BPMN отсутствует в develop)</t>
         </is>
       </c>
     </row>
@@ -510,7 +510,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Формирования документов</t>
+          <t>Подготовка документов</t>
         </is>
       </c>
     </row>
@@ -522,7 +522,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Подписание документов</t>
+          <t>Подписание</t>
         </is>
       </c>
     </row>
@@ -534,7 +534,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Оплата страховки</t>
+          <t>Оплата (stub + PT15M)</t>
         </is>
       </c>
     </row>
@@ -546,7 +546,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Финализация заявки</t>
+          <t>Финализация</t>
         </is>
       </c>
     </row>
@@ -558,7 +558,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Удаление документов</t>
+          <t>Удаление (stub)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add NT abbreviations glossary Excel
List abbreviations used in ncins NT prerequisites with full
expansions and document context.

Co-authored-by: Дмитрий Григорьев <pulya-na-vullet@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/nt-prerequisites-xlsx/00-README-index.xlsx
+++ b/nt-prerequisites-xlsx/00-README-index.xlsx
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="70" customWidth="1" min="1" max="1"/>
@@ -562,6 +562,18 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>НТ пререквизиты __ Аббревиатуры.xlsx</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>Справочник аббревиатур и расшифровок</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>